<commit_message>
Trying to take into account effect of different flow rate, but it is not changing the results of C at high C
</commit_message>
<xml_diff>
--- a/results/cal_250725_PR/nlQfittingRhoResultsAll.xlsx
+++ b/results/cal_250725_PR/nlQfittingRhoResultsAll.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="361" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="457" uniqueCount="18">
   <si>
     <t>Q</t>
   </si>
@@ -49,6 +49,24 @@
   </si>
   <si>
     <t>m</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>Q10</t>
+  </si>
+  <si>
+    <t>QAll-Hrho</t>
+  </si>
+  <si>
+    <t>QAll-Lrho</t>
   </si>
 </sst>
 </file>
@@ -94,18 +112,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="2.5703125" customWidth="true"/>
-    <col min="2" max="2" width="3.28515625" customWidth="true"/>
-    <col min="3" max="3" width="3.28515625" customWidth="true"/>
+    <col min="1" max="1" width="9.5703125" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="12.7109375" customWidth="true"/>
     <col min="4" max="4" width="3.28515625" customWidth="true"/>
     <col min="5" max="5" width="3.28515625" customWidth="true"/>
-    <col min="6" max="6" width="3.28515625" customWidth="true"/>
+    <col min="6" max="6" width="13.42578125" customWidth="true"/>
     <col min="7" max="7" width="2.85546875" customWidth="true"/>
     <col min="8" max="8" width="3.28515625" customWidth="true"/>
-    <col min="9" max="9" width="6" customWidth="true"/>
+    <col min="9" max="9" width="11.7109375" customWidth="true"/>
     <col min="10" max="10" width="5.6640625" customWidth="true"/>
   </cols>
   <sheetData>
@@ -143,121 +161,87 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B2" s="0">
-        <v>10.925162356438157</v>
+        <v>10.499442810285984</v>
       </c>
       <c r="C2" s="0">
-        <v>0.97107525751346224</v>
-      </c>
-      <c r="D2" s="0">
-        <v>0.14062457547722543</v>
-      </c>
-      <c r="E2" s="0">
-        <v>179.52813270282331</v>
-      </c>
-      <c r="F2" s="0">
-        <v>0.14946035010472461</v>
-      </c>
-      <c r="G2" s="0">
-        <v>1.1116998329906878</v>
-      </c>
-      <c r="H2" s="0">
-        <v>-25.246067447553521</v>
-      </c>
+        <v>0.97116482308278174</v>
+      </c>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
       <c r="I2" s="0">
-        <v>2.8621986961891595</v>
+        <v>2.4308386760198446</v>
       </c>
       <c r="J2" s="0">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="0"/>
+      <c r="A3" s="0" t="s">
+        <v>13</v>
+      </c>
       <c r="B3" s="0">
-        <v>0</v>
+        <v>12.150834546417428</v>
       </c>
       <c r="C3" s="0">
-        <v>0</v>
-      </c>
-      <c r="D3" s="0">
-        <v>0</v>
-      </c>
-      <c r="E3" s="0">
-        <v>0</v>
-      </c>
-      <c r="F3" s="0">
-        <v>0</v>
-      </c>
-      <c r="G3" s="0">
-        <v>0</v>
-      </c>
-      <c r="H3" s="0">
-        <v>0</v>
-      </c>
+        <v>0.96113793212425114</v>
+      </c>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
       <c r="I3" s="0">
-        <v>0</v>
+        <v>2.4308386760198446</v>
       </c>
       <c r="J3" s="0">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="0"/>
+      <c r="A4" s="0" t="s">
+        <v>14</v>
+      </c>
       <c r="B4" s="0">
-        <v>0</v>
+        <v>14.307717953329444</v>
       </c>
       <c r="C4" s="0">
-        <v>0</v>
-      </c>
-      <c r="D4" s="0">
-        <v>0</v>
-      </c>
-      <c r="E4" s="0">
-        <v>0</v>
-      </c>
-      <c r="F4" s="0">
-        <v>0</v>
-      </c>
-      <c r="G4" s="0">
-        <v>0</v>
-      </c>
-      <c r="H4" s="0">
-        <v>0</v>
-      </c>
+        <v>0.94804180583380826</v>
+      </c>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
       <c r="I4" s="0">
-        <v>0</v>
+        <v>2.4308386760198446</v>
       </c>
       <c r="J4" s="0">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="0"/>
+      <c r="A5" s="0" t="s">
+        <v>15</v>
+      </c>
       <c r="B5" s="0">
-        <v>0</v>
+        <v>15.919790761621016</v>
       </c>
       <c r="C5" s="0">
-        <v>0</v>
-      </c>
-      <c r="D5" s="0">
-        <v>0</v>
-      </c>
-      <c r="E5" s="0">
-        <v>0</v>
-      </c>
-      <c r="F5" s="0">
-        <v>0</v>
-      </c>
-      <c r="G5" s="0">
-        <v>0</v>
-      </c>
-      <c r="H5" s="0">
-        <v>0</v>
-      </c>
+        <v>0.93825365084169343</v>
+      </c>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
       <c r="I5" s="0">
-        <v>0</v>
+        <v>2.4308386760198446</v>
       </c>
       <c r="J5" s="0">
         <v>0</v>
@@ -265,34 +249,51 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="0">
-        <v>13.632775890165275</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="B6" s="0"/>
       <c r="C6" s="0">
-        <v>0.94819951587831075</v>
-      </c>
-      <c r="D6" s="0">
-        <v>0.1592975142380548</v>
-      </c>
-      <c r="E6" s="0">
-        <v>166.5546249785364</v>
-      </c>
+        <v>0.97116482308278174</v>
+      </c>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
       <c r="F6" s="0">
-        <v>0.005963208600391629</v>
-      </c>
-      <c r="G6" s="0">
-        <v>1.1074970301163656</v>
-      </c>
-      <c r="H6" s="0">
-        <v>-26.531737743932279</v>
-      </c>
+        <v>-0.014972680303354869</v>
+      </c>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
       <c r="I6" s="0">
-        <v>3.215227873919257</v>
+        <v>2.4308386760198446</v>
       </c>
       <c r="J6" s="0">
         <v>5.0076388530866272</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="0">
+        <v>13.771816002005963</v>
+      </c>
+      <c r="C7" s="0">
+        <v>0.95129568576599954</v>
+      </c>
+      <c r="D7" s="0">
+        <v>0.15960913438855961</v>
+      </c>
+      <c r="E7" s="0">
+        <v>164.69628950402301</v>
+      </c>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0">
+        <v>1.110904820154559</v>
+      </c>
+      <c r="H7" s="0">
+        <v>-12.515216202738767</v>
+      </c>
+      <c r="I7" s="0">
+        <v>3.3545980071603143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>